<commit_message>
sửa lại vòng lặp trong main về 500 và chạy lại kiểm thử
</commit_message>
<xml_diff>
--- a/results/excel_reports/Benchmark_Results.xlsx
+++ b/results/excel_reports/Benchmark_Results.xlsx
@@ -472,16 +472,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.026182457122062e-13</v>
+        <v>1.259122144390219e-14</v>
       </c>
       <c r="D2" t="n">
-        <v>2.150913293483441e-11</v>
+        <v>3.481154561286225e-11</v>
       </c>
       <c r="E2" t="n">
-        <v>3.154476809281067e-12</v>
+        <v>6.857692309507416e-12</v>
       </c>
       <c r="F2" t="n">
-        <v>4.542516978466943e-12</v>
+        <v>9.056824841030384e-12</v>
       </c>
     </row>
     <row r="3">
@@ -496,16 +496,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.467745432809114e-20</v>
+        <v>3.640714667991912e-20</v>
       </c>
       <c r="D3" t="n">
-        <v>2.019073687457035e-16</v>
+        <v>1.609179282250525e-17</v>
       </c>
       <c r="E3" t="n">
-        <v>1.330691505340854e-17</v>
+        <v>3.040815008235877e-18</v>
       </c>
       <c r="F3" t="n">
-        <v>4.146132434174666e-17</v>
+        <v>3.870765534365649e-18</v>
       </c>
     </row>
     <row r="4">
@@ -520,16 +520,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.828956611293751e-09</v>
+        <v>1.516122766338006e-09</v>
       </c>
       <c r="D4" t="n">
-        <v>5.002468857109164e-08</v>
+        <v>7.042433108325739e-08</v>
       </c>
       <c r="E4" t="n">
-        <v>1.382558912448475e-08</v>
+        <v>1.635273885695793e-08</v>
       </c>
       <c r="F4" t="n">
-        <v>1.174848835511244e-08</v>
+        <v>1.344444033543859e-08</v>
       </c>
     </row>
     <row r="5">
@@ -544,16 +544,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9.398084892130282e-13</v>
+        <v>3.958170247244982e-13</v>
       </c>
       <c r="D5" t="n">
-        <v>5.123905401258374e-11</v>
+        <v>2.004449956556242e-11</v>
       </c>
       <c r="E5" t="n">
-        <v>7.038938014762993e-12</v>
+        <v>4.943859219374888e-12</v>
       </c>
       <c r="F5" t="n">
-        <v>9.03156870839248e-12</v>
+        <v>4.027260810674818e-12</v>
       </c>
     </row>
     <row r="6">
@@ -568,16 +568,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3.410605131648481e-13</v>
+        <v>7.389644451905042e-13</v>
       </c>
       <c r="D6" t="n">
-        <v>13.43966436963535</v>
+        <v>14.82304680265548</v>
       </c>
       <c r="E6" t="n">
-        <v>3.234178443414936</v>
+        <v>1.966515466194951</v>
       </c>
       <c r="F6" t="n">
-        <v>3.610836613698035</v>
+        <v>3.814763136675019</v>
       </c>
     </row>
     <row r="7">
@@ -592,16 +592,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5.684341886080801e-14</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>21.9038391234298</v>
+        <v>75.14587695883017</v>
       </c>
       <c r="E7" t="n">
-        <v>1.771772732442048</v>
+        <v>5.712677481838169</v>
       </c>
       <c r="F7" t="n">
-        <v>4.751185929293935</v>
+        <v>14.95404878415493</v>
       </c>
     </row>
     <row r="8">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>7.515444666594817e-08</v>
+        <v>3.384206026524339e-08</v>
       </c>
       <c r="D8" t="n">
-        <v>3.891999601268736e-06</v>
+        <v>2.65607462468509e-06</v>
       </c>
       <c r="E8" t="n">
-        <v>5.09174371850681e-07</v>
+        <v>4.795780084461872e-07</v>
       </c>
       <c r="F8" t="n">
-        <v>7.89124130246399e-07</v>
+        <v>5.524197207730127e-07</v>
       </c>
     </row>
     <row r="9">
@@ -640,16 +640,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3.751354782366434e-11</v>
+        <v>2.889466443889432e-11</v>
       </c>
       <c r="D9" t="n">
-        <v>1.950873684819499e-09</v>
+        <v>2.516916897121746e-09</v>
       </c>
       <c r="E9" t="n">
-        <v>3.815931570727571e-10</v>
+        <v>3.852575443848612e-10</v>
       </c>
       <c r="F9" t="n">
-        <v>4.699884317178974e-10</v>
+        <v>4.528326268870925e-10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: - Chạy lại kiểm thử để đánh giá
</commit_message>
<xml_diff>
--- a/results/excel_reports/Benchmark_Results.xlsx
+++ b/results/excel_reports/Benchmark_Results.xlsx
@@ -472,16 +472,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.259122144390219e-14</v>
+        <v>8.583085861254752e-14</v>
       </c>
       <c r="D2" t="n">
-        <v>3.481154561286225e-11</v>
+        <v>3.006554464558929e-11</v>
       </c>
       <c r="E2" t="n">
-        <v>6.857692309507416e-12</v>
+        <v>4.165827916913464e-12</v>
       </c>
       <c r="F2" t="n">
-        <v>9.056824841030384e-12</v>
+        <v>5.798268055276131e-12</v>
       </c>
     </row>
     <row r="3">
@@ -496,16 +496,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3.640714667991912e-20</v>
+        <v>7.454045759246573e-20</v>
       </c>
       <c r="D3" t="n">
-        <v>1.609179282250525e-17</v>
+        <v>3.183176419496977e-17</v>
       </c>
       <c r="E3" t="n">
-        <v>3.040815008235877e-18</v>
+        <v>4.173826942788418e-18</v>
       </c>
       <c r="F3" t="n">
-        <v>3.870765534365649e-18</v>
+        <v>6.25995629316008e-18</v>
       </c>
     </row>
     <row r="4">
@@ -520,16 +520,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.516122766338006e-09</v>
+        <v>2.570141203129151e-09</v>
       </c>
       <c r="D4" t="n">
-        <v>7.042433108325739e-08</v>
+        <v>8.350918287548907e-08</v>
       </c>
       <c r="E4" t="n">
-        <v>1.635273885695793e-08</v>
+        <v>2.209456660053217e-08</v>
       </c>
       <c r="F4" t="n">
-        <v>1.344444033543859e-08</v>
+        <v>1.769686523810249e-08</v>
       </c>
     </row>
     <row r="5">
@@ -544,16 +544,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3.958170247244982e-13</v>
+        <v>5.518886664186726e-13</v>
       </c>
       <c r="D5" t="n">
-        <v>2.004449956556242e-11</v>
+        <v>3.262241743386641e-11</v>
       </c>
       <c r="E5" t="n">
-        <v>4.943859219374888e-12</v>
+        <v>8.559112276749595e-12</v>
       </c>
       <c r="F5" t="n">
-        <v>4.027260810674818e-12</v>
+        <v>8.524208192107588e-12</v>
       </c>
     </row>
     <row r="6">
@@ -568,16 +568,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7.389644451905042e-13</v>
+        <v>2.273736754432321e-13</v>
       </c>
       <c r="D6" t="n">
-        <v>14.82304680265548</v>
+        <v>55.99458570004725</v>
       </c>
       <c r="E6" t="n">
-        <v>1.966515466194951</v>
+        <v>6.46190005387033</v>
       </c>
       <c r="F6" t="n">
-        <v>3.814763136675019</v>
+        <v>13.85162642688278</v>
       </c>
     </row>
     <row r="7">
@@ -592,16 +592,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>1.13686837721616e-13</v>
       </c>
       <c r="D7" t="n">
-        <v>75.14587695883017</v>
+        <v>26.1655587026579</v>
       </c>
       <c r="E7" t="n">
-        <v>5.712677481838169</v>
+        <v>2.959905374533925</v>
       </c>
       <c r="F7" t="n">
-        <v>14.95404878415493</v>
+        <v>5.847365374029341</v>
       </c>
     </row>
     <row r="8">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3.384206026524339e-08</v>
+        <v>3.745380938724452e-08</v>
       </c>
       <c r="D8" t="n">
-        <v>2.65607462468509e-06</v>
+        <v>1.585019213212746e-06</v>
       </c>
       <c r="E8" t="n">
-        <v>4.795780084461872e-07</v>
+        <v>2.98139545377533e-07</v>
       </c>
       <c r="F8" t="n">
-        <v>5.524197207730127e-07</v>
+        <v>2.742600127483084e-07</v>
       </c>
     </row>
     <row r="9">
@@ -640,16 +640,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2.889466443889432e-11</v>
+        <v>3.577982354840969e-11</v>
       </c>
       <c r="D9" t="n">
-        <v>2.516916897121746e-09</v>
+        <v>2.083674122133061e-09</v>
       </c>
       <c r="E9" t="n">
-        <v>3.852575443848612e-10</v>
+        <v>3.955215710504945e-10</v>
       </c>
       <c r="F9" t="n">
-        <v>4.528326268870925e-10</v>
+        <v>4.548763604419862e-10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>